<commit_message>
A2-3 Werner: Literaturverzeichnis korrigiert (References, Zitierschlüssel, EURO23/PLAZ23 vollständig)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
+++ b/#zusätzliche_daten/gi-dl-datacite-dublincore-metadata.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" tabRatio="216" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5460" yWindow="2250" windowWidth="27920" windowHeight="9960" tabRatio="216" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelle1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,20 +51,13 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -75,12 +68,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,47 +85,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -487,149 +461,150 @@
   <dimension ref="A1:V15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5"/>
   <cols>
-    <col width="40.83203125" customWidth="1" style="5" min="1" max="1"/>
-    <col width="48.33203125" customWidth="1" style="5" min="2" max="2"/>
-    <col width="10.83203125" customWidth="1" style="5" min="3" max="3"/>
-    <col width="14" customWidth="1" style="5" min="4" max="4"/>
-    <col width="23.4140625" customWidth="1" style="5" min="5" max="5"/>
-    <col width="24.33203125" customWidth="1" style="5" min="6" max="7"/>
-    <col width="8.33203125" customWidth="1" style="5" min="8" max="8"/>
-    <col width="7.25" customWidth="1" style="7" min="9" max="9"/>
-    <col width="29.9140625" customWidth="1" style="5" min="10" max="10"/>
-    <col width="10.6640625" customWidth="1" style="5" min="11" max="12"/>
-    <col width="24.9140625" customWidth="1" style="5" min="13" max="13"/>
-    <col width="14.58203125" customWidth="1" style="5" min="14" max="14"/>
-    <col width="10.6640625" customWidth="1" style="5" min="15" max="15"/>
-    <col width="8.9140625" customWidth="1" style="5" min="16" max="16"/>
-    <col width="20" customWidth="1" style="5" min="17" max="17"/>
-    <col width="22.6640625" customWidth="1" style="5" min="18" max="18"/>
-    <col width="37.33203125" customWidth="1" style="5" min="19" max="19"/>
-    <col width="19.58203125" customWidth="1" style="5" min="20" max="20"/>
-    <col width="19.6640625" customWidth="1" style="5" min="21" max="21"/>
-    <col width="26.33203125" customWidth="1" style="5" min="22" max="22"/>
-    <col width="10.6640625" customWidth="1" style="5" min="23" max="16384"/>
+    <col width="40.83203125" customWidth="1" style="4" min="1" max="1"/>
+    <col width="48.33203125" customWidth="1" style="4" min="2" max="2"/>
+    <col width="10.83203125" customWidth="1" style="4" min="3" max="3"/>
+    <col width="14" customWidth="1" style="4" min="4" max="4"/>
+    <col width="23.4140625" customWidth="1" style="4" min="5" max="5"/>
+    <col width="24.33203125" customWidth="1" style="4" min="6" max="7"/>
+    <col width="8.33203125" customWidth="1" style="4" min="8" max="8"/>
+    <col width="7.25" customWidth="1" style="6" min="9" max="9"/>
+    <col width="29.9140625" customWidth="1" style="4" min="10" max="10"/>
+    <col width="10.6640625" customWidth="1" style="4" min="11" max="12"/>
+    <col width="24.9140625" customWidth="1" style="4" min="13" max="13"/>
+    <col width="14.58203125" customWidth="1" style="4" min="14" max="14"/>
+    <col width="10.6640625" customWidth="1" style="4" min="15" max="15"/>
+    <col width="8.9140625" customWidth="1" style="4" min="16" max="16"/>
+    <col width="20" customWidth="1" style="4" min="17" max="17"/>
+    <col width="22.6640625" customWidth="1" style="4" min="18" max="18"/>
+    <col width="37.33203125" customWidth="1" style="4" min="19" max="19"/>
+    <col width="19.58203125" customWidth="1" style="4" min="20" max="20"/>
+    <col width="19.6640625" customWidth="1" style="4" min="21" max="21"/>
+    <col width="26.33203125" customWidth="1" style="4" min="22" max="22"/>
+    <col width="10.6640625" customWidth="1" style="4" min="23" max="23"/>
+    <col width="10.6640625" customWidth="1" style="4" min="24" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="61.5" customFormat="1" customHeight="1" s="8">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="61.5" customFormat="1" customHeight="1" s="7">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>dc.title</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>dc.contributor.author</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>dc.language.iso</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>dc.relation.ispartof</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>dc.contributor.editor</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>dc.relation.ispartofseries</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>dc.publisher</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>gi.citation.publisherPlace</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>dc.date.issued</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>dc.description.abstract</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>dc.subject</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>gi.tag</t>
         </is>
       </c>
-      <c r="M1" s="8" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>dc.identifier.doi</t>
         </is>
       </c>
-      <c r="N1" s="8" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>dc.identifier.pissn</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>gi.citation.startPage</t>
         </is>
       </c>
-      <c r="P1" s="8" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>gi.citation.endPage</t>
         </is>
       </c>
-      <c r="Q1" s="8" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>gi.conference.date</t>
         </is>
       </c>
-      <c r="R1" s="8" t="inlineStr">
+      <c r="R1" s="7" t="inlineStr">
         <is>
           <t>gi.conference.location</t>
         </is>
       </c>
-      <c r="S1" s="8" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>gi.conference.sessiontitle</t>
         </is>
       </c>
-      <c r="T1" s="8" t="inlineStr">
+      <c r="T1" s="7" t="inlineStr">
         <is>
           <t>dc.type</t>
         </is>
       </c>
-      <c r="U1" s="8" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>gi.conference.review</t>
         </is>
       </c>
-      <c r="V1" s="8" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>filename</t>
         </is>
       </c>
     </row>
-    <row r="2" customFormat="1" s="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" customFormat="1" s="1">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>nachfolgend ein paar Beispieldaten:</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14" customFormat="1" customHeight="1" s="1">
+    <row r="3" ht="14" customFormat="1" customHeight="1" s="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>Web-based management and analysis of nature conservation measures in Schleswig-Holstein – current developments</t>
@@ -730,7 +705,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="4" ht="15" customFormat="1" customHeight="1" s="3">
       <c r="A4" t="inlineStr">
         <is>
           <t>Common and Domain-Specific Design Patterns for Mobile AR Applications to Visualize Measures on Building Facades in an Environmental Context</t>
@@ -831,7 +806,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customFormat="1" customHeight="1" s="5">
+    <row r="5" ht="17" customHeight="1" s="2">
       <c r="A5" t="inlineStr">
         <is>
           <t>Sustainability Context Inheritance: From Trusted Evidence to Product Sustainability Profiles in Circular Economy Decision-Making</t>
@@ -932,7 +907,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customFormat="1" customHeight="1" s="5">
+    <row r="6" ht="16" customHeight="1" s="2">
       <c r="A6" t="inlineStr">
         <is>
           <t>AI model of a photovoltaic installation</t>
@@ -1033,7 +1008,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customFormat="1" customHeight="1" s="5">
+    <row r="7" ht="16" customHeight="1" s="2">
       <c r="A7" t="inlineStr">
         <is>
           <t>Environmentally Informed GenAI Use in ITSM: A Problem Analysis of Organisational Use-Case Decision-Making</t>
@@ -1134,7 +1109,7 @@
         </is>
       </c>
     </row>
-    <row r="8" customFormat="1" s="5">
+    <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>Application of Artificial Intelligence in German Municipal Wastewater Facilities</t>
@@ -1235,7 +1210,7 @@
         </is>
       </c>
     </row>
-    <row r="9" customFormat="1" s="6">
+    <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>Assessing the Maturity of Sustainability-aware Data Management Strategies that minimise Data Volumes and reduce Energy Consumption: A Study Approach</t>
@@ -1336,7 +1311,7 @@
         </is>
       </c>
     </row>
-    <row r="10" customFormat="1" s="5">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>Linking Water Quality to Corrosion Behaviour at Steel Sheet Pile Walls: A Machine Learning Study in the Port of Hamburg</t>
@@ -1437,7 +1412,7 @@
         </is>
       </c>
     </row>
-    <row r="11" customFormat="1" s="6">
+    <row r="11">
       <c r="A11" t="inlineStr">
         <is>
           <t>Air Quality Knowledge as a Driver of Computing Competences: An International Project-Based Learning Project</t>
@@ -1538,7 +1513,7 @@
         </is>
       </c>
     </row>
-    <row r="12" customFormat="1" s="5">
+    <row r="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>Windows Integration into the Green Metrics Tool: Energy Measurement of Native Windows Applications via RAPL</t>
@@ -1639,7 +1614,7 @@
         </is>
       </c>
     </row>
-    <row r="13" customFormat="1" s="5">
+    <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t>Joint Evaluation of the Green Coding Roadmap Training</t>
@@ -1740,7 +1715,7 @@
         </is>
       </c>
     </row>
-    <row r="14" customFormat="1" s="5">
+    <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>Toward a Framework for Performance and Carbon Footprint Assessment of Payment Channel Network Solutions</t>
@@ -1841,7 +1816,7 @@
         </is>
       </c>
     </row>
-    <row r="15" customFormat="1" s="5">
+    <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>Towards a Taxonomy of ICT and Software Sustainability Assessment Instruments</t>
@@ -1942,19 +1917,19 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="306" customFormat="1" customHeight="1" s="11"/>
-    <row r="26" customFormat="1" s="5"/>
-    <row r="27" customFormat="1" s="5"/>
-    <row r="28" customFormat="1" s="5"/>
-    <row r="29" customFormat="1" s="5"/>
-    <row r="30" customFormat="1" s="5"/>
-    <row r="31" customFormat="1" s="5"/>
-    <row r="32" customFormat="1" s="5"/>
-    <row r="33" customFormat="1" s="5"/>
-    <row r="34" customFormat="1" s="5"/>
-    <row r="35" customFormat="1" s="5"/>
-    <row r="36" customFormat="1" s="5"/>
-    <row r="37" customFormat="1" s="5"/>
+    <row r="25" ht="306" customFormat="1" customHeight="1" s="5"/>
+    <row r="26" customFormat="1" s="4"/>
+    <row r="27" customFormat="1" s="4"/>
+    <row r="28" customFormat="1" s="4"/>
+    <row r="29" customFormat="1" s="4"/>
+    <row r="30" customFormat="1" s="4"/>
+    <row r="31" customFormat="1" s="4"/>
+    <row r="32" customFormat="1" s="4"/>
+    <row r="33" customFormat="1" s="4"/>
+    <row r="34" customFormat="1" s="4"/>
+    <row r="35" customFormat="1" s="4"/>
+    <row r="36" customFormat="1" s="4"/>
+    <row r="37" customFormat="1" s="4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>